<commit_message>
FEASIBLE SOLUTION ACHIEVED! -  Iterative Manual Assignment
</commit_message>
<xml_diff>
--- a/Decision_analytics/Module6/Manual District Reassignment.xlsx
+++ b/Decision_analytics/Module6/Manual District Reassignment.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefanjenss/Desktop/DataScience/Decision_analytics/Module6/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C217CC-31B3-694B-8A32-D47620EE26D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFEF6458-970B-304C-B738-00E7C0743354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16060" xr2:uid="{44453298-CD55-E24A-8C56-71665D6DF46C}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="19580" xr2:uid="{44453298-CD55-E24A-8C56-71665D6DF46C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
   <si>
     <t>All Counties</t>
   </si>
@@ -315,13 +315,26 @@
   </si>
   <si>
     <t>Potentially add more to get the number closer to 564,400</t>
+  </si>
+  <si>
+    <t>District 9</t>
+  </si>
+  <si>
+    <t>District 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -345,8 +358,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -356,6 +376,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -369,19 +395,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -432,28 +471,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EC0F823D-7113-F240-B124-5E5C25F203CF}" name="Table1" displayName="Table1" ref="A1:B107" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EC0F823D-7113-F240-B124-5E5C25F203CF}" name="Table1" displayName="Table1" ref="A1:B107" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:B107" xr:uid="{EC0F823D-7113-F240-B124-5E5C25F203CF}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B107">
-    <sortCondition ref="A1:A107"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B51">
+    <sortCondition descending="1" ref="B1:B107"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{1FACA074-0481-B84F-9BBE-F94F3262215E}" name="All Counties"/>
-    <tableColumn id="2" xr3:uid="{2B535D85-C4A5-CA4A-BD30-56B8C264A4BE}" name="Population"/>
+    <tableColumn id="2" xr3:uid="{2B535D85-C4A5-CA4A-BD30-56B8C264A4BE}" name="Population" dataDxfId="1" dataCellStyle="Comma"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{190D87A8-6FEC-AD48-B03C-4A2D6C9F47A3}" name="Table2" displayName="Table2" ref="D1:E25" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{190D87A8-6FEC-AD48-B03C-4A2D6C9F47A3}" name="Table2" displayName="Table2" ref="D1:E25" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="D1:E25" xr:uid="{190D87A8-6FEC-AD48-B03C-4A2D6C9F47A3}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D2:E25">
     <sortCondition ref="D1:D25"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A2006382-096E-904A-A322-2018E8DFA596}" name="District 11 (Northern)"/>
-    <tableColumn id="2" xr3:uid="{11BE992F-B0D5-6C49-B144-FC59BF9140BA}" name="Population"/>
+    <tableColumn id="2" xr3:uid="{11BE992F-B0D5-6C49-B144-FC59BF9140BA}" name="Population" dataDxfId="0" dataCellStyle="Comma"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -756,27 +795,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B82318-DBB4-3A4B-96CF-365FC71DBEAD}">
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="13.1640625" style="6" customWidth="1"/>
     <col min="3" max="3" width="5.83203125" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>84</v>
       </c>
       <c r="D1" s="2" t="s">
@@ -788,13 +827,13 @@
       <c r="G1" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="7" t="s">
         <v>84</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="7" t="s">
         <v>84</v>
       </c>
       <c r="M1" s="2" t="s">
@@ -806,27 +845,27 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B2">
-        <v>10417</v>
+        <v>50</v>
+      </c>
+      <c r="B2" s="6">
+        <v>366376</v>
       </c>
       <c r="D2" t="s">
         <v>26</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="6">
         <v>8807</v>
       </c>
       <c r="G2" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="5">
         <v>874195</v>
       </c>
       <c r="J2" t="s">
         <v>68</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="5">
         <v>1269431</v>
       </c>
       <c r="M2" t="s">
@@ -838,597 +877,603 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B3">
-        <v>121210</v>
+        <v>17</v>
+      </c>
+      <c r="B3" s="6">
+        <v>300873</v>
       </c>
       <c r="D3" t="s">
         <v>47</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="6">
         <v>28847</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4">
-        <v>15089</v>
+        <v>52</v>
+      </c>
+      <c r="B4" s="6">
+        <v>284108</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="6">
         <v>24249</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="K4" s="8" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5">
-        <v>63554</v>
+        <v>51</v>
+      </c>
+      <c r="B5" s="6">
+        <v>261173</v>
       </c>
       <c r="D5" t="s">
         <v>75</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="6">
         <v>8277</v>
       </c>
       <c r="G5" t="s">
         <v>1</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="6">
         <v>22870</v>
+      </c>
+      <c r="J5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" s="6">
+        <v>659083</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6">
-        <v>102821</v>
+        <v>14</v>
+      </c>
+      <c r="B6" s="6">
+        <v>188330</v>
       </c>
       <c r="D6" t="s">
         <v>81</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="6">
         <v>26293</v>
       </c>
       <c r="G6" t="s">
         <v>55</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="6">
         <v>18297</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7">
-        <v>152900</v>
+        <v>72</v>
+      </c>
+      <c r="B7" s="6">
+        <v>176565</v>
       </c>
       <c r="D7" t="s">
         <v>61</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="6">
         <v>25940</v>
       </c>
       <c r="G7" t="s">
         <v>33</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="6">
         <v>25287</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8">
-        <v>44531</v>
+        <v>11</v>
+      </c>
+      <c r="B8" s="6">
+        <v>160151</v>
       </c>
       <c r="D8" t="s">
         <v>63</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="6">
         <v>36293</v>
       </c>
       <c r="G8" t="s">
         <v>66</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="6">
         <v>29409</v>
+      </c>
+      <c r="J8" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="6">
+        <v>401983</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9">
-        <v>133289</v>
+        <v>32</v>
+      </c>
+      <c r="B9" s="6">
+        <v>160066</v>
       </c>
       <c r="D9" t="s">
         <v>76</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="6">
         <v>36741</v>
       </c>
       <c r="G9" t="s">
         <v>3</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="6">
         <v>34196</v>
+      </c>
+      <c r="J9" t="s">
+        <v>83</v>
+      </c>
+      <c r="K9" s="6">
+        <v>196161</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10">
-        <v>51403</v>
+        <v>69</v>
+      </c>
+      <c r="B10" s="6">
+        <v>155609</v>
       </c>
       <c r="D10" t="s">
         <v>53</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="6">
         <v>25874</v>
       </c>
       <c r="G10" t="s">
         <v>64</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="6">
         <v>12594</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K10" s="6">
+        <f>SUM(K8:K9)</f>
+        <v>598144</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B11">
-        <v>79748</v>
+        <v>18</v>
+      </c>
+      <c r="B11" s="6">
+        <v>152900</v>
       </c>
       <c r="D11" t="s">
         <v>29</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="6">
         <v>34163</v>
       </c>
       <c r="G11" t="s">
         <v>74</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="6">
         <v>96464</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12">
-        <v>13491</v>
+        <v>34</v>
+      </c>
+      <c r="B12" s="6">
+        <v>133289</v>
       </c>
       <c r="D12" t="s">
         <v>39</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="6">
         <v>14319</v>
       </c>
       <c r="G12" t="s">
         <v>23</v>
       </c>
-      <c r="H12">
+      <c r="H12" s="6">
         <v>50886</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>62</v>
-      </c>
-      <c r="B13">
-        <v>108992</v>
+        <v>70</v>
+      </c>
+      <c r="B13" s="6">
+        <v>121210</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="6">
         <v>37035</v>
       </c>
       <c r="G13" t="s">
         <v>12</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="6">
         <v>15213</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B14">
-        <v>401983</v>
+        <v>62</v>
+      </c>
+      <c r="B14" s="6">
+        <v>108992</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="6">
         <v>11622</v>
       </c>
       <c r="G14" t="s">
         <v>30</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="6">
         <v>23274</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15">
-        <v>25728</v>
+        <v>54</v>
+      </c>
+      <c r="B15" s="6">
+        <v>102821</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="6">
         <v>2180</v>
       </c>
       <c r="G15" t="s">
         <v>6</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="6">
         <v>40720</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>73</v>
-      </c>
-      <c r="B16">
-        <v>41100</v>
+        <v>22</v>
+      </c>
+      <c r="B16" s="6">
+        <v>98567</v>
       </c>
       <c r="D16" t="s">
         <v>58</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="6">
         <v>5330</v>
       </c>
       <c r="G16" t="s">
         <v>57</v>
       </c>
-      <c r="H16">
+      <c r="H16" s="6">
         <v>31352</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17">
-        <v>45762</v>
+        <v>79</v>
+      </c>
+      <c r="B17" s="6">
+        <v>88780</v>
       </c>
       <c r="D17" t="s">
         <v>67</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="6">
         <v>10941</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="H17">
-        <f>SUM(H5:H16)</f>
-        <v>400562</v>
+      <c r="G17" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" s="6">
+        <v>18182</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18">
-        <v>31248</v>
+        <v>41</v>
+      </c>
+      <c r="B18" s="6">
+        <v>83674</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="6">
         <v>66661</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>92</v>
+      <c r="G18" t="s">
+        <v>45</v>
+      </c>
+      <c r="H18" s="6">
+        <v>26973</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19">
-        <v>284108</v>
+        <v>2</v>
+      </c>
+      <c r="B19" s="6">
+        <v>79748</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="6">
         <v>23266</v>
+      </c>
+      <c r="G19" t="s">
+        <v>10</v>
+      </c>
+      <c r="H19" s="6">
+        <v>13491</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20">
-        <v>66809</v>
+        <v>16</v>
+      </c>
+      <c r="B20" s="6">
+        <v>75692</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="6">
         <v>9569</v>
+      </c>
+      <c r="G20" t="s">
+        <v>24</v>
+      </c>
+      <c r="H20" s="6">
+        <v>23708</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21">
-        <v>25521</v>
+        <v>20</v>
+      </c>
+      <c r="B21" s="6">
+        <v>68022</v>
       </c>
       <c r="D21" t="s">
         <v>38</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="6">
         <v>5863</v>
+      </c>
+      <c r="G21" t="s">
+        <v>8</v>
+      </c>
+      <c r="H21" s="6">
+        <v>64447</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22">
-        <v>64447</v>
+        <v>60</v>
+      </c>
+      <c r="B22" s="6">
+        <v>67433</v>
       </c>
       <c r="D22" t="s">
         <v>21</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="6">
         <v>25644</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H22" s="6">
+        <f>SUM(H5:H21)</f>
+        <v>547363</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23">
-        <v>160066</v>
+        <v>5</v>
+      </c>
+      <c r="B23" s="6">
+        <v>66809</v>
       </c>
       <c r="D23" t="s">
         <v>85</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="6">
         <v>13361</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24">
-        <v>261173</v>
+        <v>28</v>
+      </c>
+      <c r="B24" s="6">
+        <v>63554</v>
       </c>
       <c r="D24" t="s">
         <v>9</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="6">
         <v>8188</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>65</v>
-      </c>
-      <c r="B25">
-        <v>18182</v>
+        <v>43</v>
+      </c>
+      <c r="B25" s="6">
+        <v>60874</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="5">
         <f>SUM(E2:E24)</f>
         <v>489463</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>42</v>
-      </c>
-      <c r="B26">
-        <v>659083</v>
+        <v>35</v>
+      </c>
+      <c r="B26" s="6">
+        <v>52945</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>79</v>
-      </c>
-      <c r="B27">
-        <v>88780</v>
+        <v>78</v>
+      </c>
+      <c r="B27" s="6">
+        <v>51403</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28">
-        <v>98567</v>
+        <v>77</v>
+      </c>
+      <c r="B28" s="6">
+        <v>45762</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>83</v>
-      </c>
-      <c r="B29">
-        <v>196161</v>
+        <v>4</v>
+      </c>
+      <c r="B29" s="6">
+        <v>44531</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>41</v>
-      </c>
-      <c r="B30">
-        <v>83674</v>
+        <v>73</v>
+      </c>
+      <c r="B30" s="6">
+        <v>41100</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31">
-        <v>155609</v>
+        <v>48</v>
+      </c>
+      <c r="B31" s="6">
+        <v>40657</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B32">
-        <v>67433</v>
+        <v>56</v>
+      </c>
+      <c r="B32" s="6">
+        <v>31248</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33">
-        <v>176565</v>
+        <v>36</v>
+      </c>
+      <c r="B33" s="6">
+        <v>25728</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>45</v>
-      </c>
-      <c r="B34">
-        <v>26973</v>
+        <v>46</v>
+      </c>
+      <c r="B34" s="6">
+        <v>25521</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>44</v>
       </c>
-      <c r="B35">
+      <c r="B35" s="6">
         <v>20970</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36">
-        <v>8404</v>
+        <v>80</v>
+      </c>
+      <c r="B36" s="6">
+        <v>15089</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>17</v>
-      </c>
-      <c r="B37">
-        <v>300873</v>
+        <v>13</v>
+      </c>
+      <c r="B37" s="6">
+        <v>13361</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>13</v>
-      </c>
-      <c r="B38">
-        <v>13361</v>
+        <v>82</v>
+      </c>
+      <c r="B38" s="6">
+        <v>10417</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>24</v>
-      </c>
-      <c r="B39">
-        <v>23708</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>14</v>
-      </c>
-      <c r="B40">
-        <v>188330</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41">
-        <v>40657</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>20</v>
-      </c>
-      <c r="B42">
-        <v>68022</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43">
-        <v>160151</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>43</v>
-      </c>
-      <c r="B44">
-        <v>60874</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>35</v>
-      </c>
-      <c r="B45">
-        <v>52945</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46">
-        <v>75692</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47">
-        <v>366376</v>
+        <v>49</v>
+      </c>
+      <c r="B39" s="6">
+        <v>8404</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  <conditionalFormatting sqref="G23 A3:A6 J5 A1 A8:A11 A13:A17 A19:A21 A23:A24 G20:G21 A26:A29 A31 A34 G5:G6 A40:A42 A44 A47:A58 A60:A61 G8:G18 A63:A107 M2 J2 G2">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A6 A8:A11 A13:A17 A19:A29 A31 A33:A34 G5:G6 A38 A40:A42 A44 A47:A58 A60:A61 G8:G16 A63:A107 M2 J2 G2 G18">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="J5">
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">

</xml_diff>